<commit_message>
Updated UAT Pack, Added CR closed document, updated README file
</commit_message>
<xml_diff>
--- a/docs/v2/04_SDT_V2_Production_UAT_Pack.xlsx
+++ b/docs/v2/04_SDT_V2_Production_UAT_Pack.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="UAT Summary" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="301">
   <si>
     <t xml:space="preserve">SDT V2 - Production User Acceptance Testing (UAT) Pack</t>
   </si>
@@ -312,35 +312,8 @@
     <t xml:space="preserve">Blank page, 404/500 error, configuration error, or application fails to render.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">App/website loads properly @ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://self-development-tracker-sdt.vercel.app/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.
+    <t xml:space="preserve">App/website loads properly @ https://self-development-tracker-sdt.vercel.app/.
 Authentication screen correctly appears.</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">Pass</t>
@@ -390,7 +363,7 @@
     <t xml:space="preserve">Login page is open</t>
   </si>
   <si>
-    <t xml:space="preserve">Email: uat.sdt.user1@example.com
+    <t xml:space="preserve">Email: sdt.user1@example.com
 Password: deliberately incorrect password</t>
   </si>
   <si>
@@ -1007,6 +980,9 @@
     <t xml:space="preserve">SDT V2 - UAT Defect Log</t>
   </si>
   <si>
+    <t xml:space="preserve">No defects identified during Production UAT </t>
+  </si>
+  <si>
     <t xml:space="preserve">Related Test Case</t>
   </si>
   <si>
@@ -1025,9 +1001,6 @@
     <t xml:space="preserve">Resolution / Retest Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">Open</t>
-  </si>
-  <si>
     <t xml:space="preserve">SDT V2 - Production UAT Sign-Off</t>
   </si>
   <si>
@@ -1040,7 +1013,7 @@
     <t xml:space="preserve">Date</t>
   </si>
   <si>
-    <t xml:space="preserve">10 October 2026</t>
+    <t xml:space="preserve">3 October 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Decision</t>
@@ -1203,7 +1176,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1237,6 +1210,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1501,26 +1482,6 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="UATDefects" displayName="UATDefects" ref="A3:L28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <tableColumns count="12">
-    <tableColumn id="1" name="Defect ID"/>
-    <tableColumn id="2" name="Related Test Case"/>
-    <tableColumn id="3" name="Date Raised"/>
-    <tableColumn id="4" name="Summary"/>
-    <tableColumn id="5" name="Steps / Context"/>
-    <tableColumn id="6" name="Expected Result"/>
-    <tableColumn id="7" name="Actual Result"/>
-    <tableColumn id="8" name="Severity"/>
-    <tableColumn id="9" name="Priority"/>
-    <tableColumn id="10" name="Status"/>
-    <tableColumn id="11" name="Owner"/>
-    <tableColumn id="12" name="Resolution / Retest Notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChatGPT">
   <a:themeElements>
@@ -2223,7 +2184,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2329,7 +2290,7 @@
       <c r="I5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="9" t="s">
         <v>95</v>
       </c>
       <c r="K5" s="4" t="s">
@@ -3359,7 +3320,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="J5" r:id="rId1" display="https://self-development-tracker-sdt.vercel.app/"/>
+    <hyperlink ref="J5" r:id="rId1" display="App/website loads properly @ https://self-development-tracker-sdt.vercel.app/.&#10;Authentication screen correctly appears."/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3379,10 +3340,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
@@ -3409,21 +3370,26 @@
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
     </row>
+    <row r="2" customFormat="false" ht="24.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>284</v>
+      </c>
+    </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
         <v>86</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>83</v>
@@ -3432,7 +3398,7 @@
         <v>85</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>26</v>
@@ -3444,527 +3410,38 @@
         <v>29</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J26" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J27" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J28" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-    </row>
+    </row>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H4:H28" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I4:I28" type="list">
-      <formula1>"Critical,High,Medium,Low"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J4:J28" type="list">
-      <formula1>"Open,In Progress,Ready for Retest,Closed,Deferred"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3972,9 +3449,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <tableParts>
-    <tablePart r:id="rId1"/>
-  </tableParts>
+  <tableParts/>
 </worksheet>
 </file>
 

</xml_diff>